<commit_message>
Fix Vencidos depot mapping from 0009 to 0099 (v1.8.103).
Acerto Inventário / sem FI / Emitir doc and recon now link Unilog class 104 to SAP depot 0099.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/mapa_acertos_template.xlsx
+++ b/assets/mapa_acertos_template.xlsx
@@ -13,7 +13,7 @@
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="884" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="0009" sheetId="42" r:id="rId1"/>
+    <sheet name="0099" sheetId="42" r:id="rId1"/>
     <sheet name="0044" sheetId="41" r:id="rId2"/>
     <sheet name="0008" sheetId="40" r:id="rId3"/>
     <sheet name="0022" sheetId="39" r:id="rId4"/>
@@ -21,32 +21,32 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'0008'!$A$9:$N$129</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'0009'!$A$9:$N$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'0099'!$A$9:$N$129</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'0011'!$A$9:$N$129</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'0022'!$A$9:$N$129</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'0044'!$A$9:$N$129</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'0008'!$A$1:$O$129</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'0009'!$A$1:$O$129</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'0099'!$A$1:$O$129</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'0011'!$A$1:$O$129</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'0022'!$A$1:$O$129</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'0044'!$A$1:$O$129</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'0008'!$1:$9</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'0009'!$1:$9</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'0099'!$1:$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'0011'!$1:$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'0022'!$1:$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'0044'!$1:$9</definedName>
     <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.Cols" localSheetId="2" hidden="1">'0008'!#REF!,'0008'!#REF!</definedName>
-    <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.Cols" localSheetId="0" hidden="1">'0009'!#REF!,'0009'!#REF!</definedName>
+    <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.Cols" localSheetId="0" hidden="1">'0099'!#REF!,'0099'!#REF!</definedName>
     <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.Cols" localSheetId="4" hidden="1">'0011'!#REF!,'0011'!#REF!</definedName>
     <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.Cols" localSheetId="3" hidden="1">'0022'!#REF!,'0022'!#REF!</definedName>
     <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.Cols" localSheetId="1" hidden="1">'0044'!#REF!,'0044'!#REF!</definedName>
     <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.PrintArea" localSheetId="2" hidden="1">'0008'!$A$1:$M$128</definedName>
-    <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.PrintArea" localSheetId="0" hidden="1">'0009'!$A$1:$M$128</definedName>
+    <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.PrintArea" localSheetId="0" hidden="1">'0099'!$A$1:$M$128</definedName>
     <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.PrintArea" localSheetId="4" hidden="1">'0011'!$A$1:$M$128</definedName>
     <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.PrintArea" localSheetId="3" hidden="1">'0022'!$A$1:$M$128</definedName>
     <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.PrintArea" localSheetId="1" hidden="1">'0044'!$A$1:$M$128</definedName>
     <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.PrintTitles" localSheetId="2" hidden="1">'0008'!$7:$8</definedName>
-    <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.PrintTitles" localSheetId="0" hidden="1">'0009'!$7:$8</definedName>
+    <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.PrintTitles" localSheetId="0" hidden="1">'0099'!$7:$8</definedName>
     <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.PrintTitles" localSheetId="4" hidden="1">'0011'!$7:$8</definedName>
     <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.PrintTitles" localSheetId="3" hidden="1">'0022'!$7:$8</definedName>
     <definedName name="Z_CFE7CC00_9D22_11D3_A09D_0050044DA93D_.wvu.PrintTitles" localSheetId="1" hidden="1">'0044'!$7:$8</definedName>

</xml_diff>